<commit_message>
Fix bugs identified during code review
Co-authored-by: google-labs-jules[bot] <161369871+google-labs-jules[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/gas_project/CSDL_DaoTaoNghe_Template.xlsx
+++ b/gas_project/CSDL_DaoTaoNghe_Template.xlsx
@@ -887,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -958,6 +958,23 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NamHienTai</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Năm mặc định khi tạo khóa học</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>